<commit_message>
data(nzd): monthly refresh 2026-09-19T08:37Z
</commit_message>
<xml_diff>
--- a/logs/nzd/raw/D30.xlsx
+++ b/logs/nzd/raw/D30.xlsx
@@ -30484,6 +30484,219 @@
         <v>16</v>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" s="28">
+        <v>46265</v>
+      </c>
+      <c r="B139" s="16">
+        <v>237495</v>
+      </c>
+      <c r="C139" s="16">
+        <v>207410</v>
+      </c>
+      <c r="D139" s="16">
+        <v>75630</v>
+      </c>
+      <c r="E139" s="16">
+        <v>16111</v>
+      </c>
+      <c r="F139" s="16">
+        <v>40226</v>
+      </c>
+      <c r="G139" s="16">
+        <v>64</v>
+      </c>
+      <c r="H139" s="16">
+        <v>11238</v>
+      </c>
+      <c r="I139"/>
+      <c r="J139" s="16">
+        <v>492</v>
+      </c>
+      <c r="K139" s="16">
+        <v>6</v>
+      </c>
+      <c r="L139" s="16">
+        <v>689</v>
+      </c>
+      <c r="M139" s="16">
+        <v>119286</v>
+      </c>
+      <c r="N139" s="16">
+        <v>5</v>
+      </c>
+      <c r="O139" s="16">
+        <v>1415</v>
+      </c>
+      <c r="P139" s="16">
+        <v>10387</v>
+      </c>
+      <c r="Q139" s="16">
+        <v>19493</v>
+      </c>
+      <c r="R139" s="16">
+        <v>4124</v>
+      </c>
+      <c r="S139" s="16">
+        <v>1400</v>
+      </c>
+      <c r="T139" s="16">
+        <v>241</v>
+      </c>
+      <c r="U139" s="16">
+        <v>1</v>
+      </c>
+      <c r="V139" s="16">
+        <v>11190</v>
+      </c>
+      <c r="W139"/>
+      <c r="X139" s="16">
+        <v>1</v>
+      </c>
+      <c r="Y139"/>
+      <c r="Z139" s="16">
+        <v>35</v>
+      </c>
+      <c r="AA139" s="16">
+        <v>4142</v>
+      </c>
+      <c r="AB139" s="16">
+        <v>0</v>
+      </c>
+      <c r="AC139" s="16">
+        <v>134</v>
+      </c>
+      <c r="AD139" s="16">
+        <v>339</v>
+      </c>
+      <c r="AE139" s="16">
+        <v>4790</v>
+      </c>
+      <c r="AF139" s="16">
+        <v>3734</v>
+      </c>
+      <c r="AG139" s="16">
+        <v>0</v>
+      </c>
+      <c r="AH139" s="16">
+        <v>3460</v>
+      </c>
+      <c r="AI139" s="16">
+        <v>35</v>
+      </c>
+      <c r="AJ139"/>
+      <c r="AK139"/>
+      <c r="AL139"/>
+      <c r="AM139"/>
+      <c r="AN139" s="16">
+        <v>1021</v>
+      </c>
+      <c r="AO139" s="16">
+        <v>0</v>
+      </c>
+      <c r="AP139" s="16">
+        <v>152</v>
+      </c>
+      <c r="AQ139" s="16">
+        <v>137</v>
+      </c>
+      <c r="AR139" s="16">
+        <v>1</v>
+      </c>
+      <c r="AS139" s="16">
+        <v>1</v>
+      </c>
+      <c r="AT139"/>
+      <c r="AU139"/>
+      <c r="AV139"/>
+      <c r="AW139" s="16">
+        <v>135</v>
+      </c>
+      <c r="AX139" s="16">
+        <v>1</v>
+      </c>
+      <c r="AY139" s="16">
+        <v>5665</v>
+      </c>
+      <c r="AZ139" s="16">
+        <v>3723</v>
+      </c>
+      <c r="BA139" s="16">
+        <v>1846</v>
+      </c>
+      <c r="BB139" s="16">
+        <v>8</v>
+      </c>
+      <c r="BC139" s="16">
+        <v>325</v>
+      </c>
+      <c r="BD139" s="16">
+        <v>405</v>
+      </c>
+      <c r="BE139" s="16">
+        <v>2</v>
+      </c>
+      <c r="BF139" s="16">
+        <v>293</v>
+      </c>
+      <c r="BG139" s="16">
+        <v>905</v>
+      </c>
+      <c r="BH139" s="16">
+        <v>3</v>
+      </c>
+      <c r="BI139" s="16">
+        <v>45</v>
+      </c>
+      <c r="BJ139" s="16">
+        <v>219984</v>
+      </c>
+      <c r="BK139" s="16">
+        <v>191299</v>
+      </c>
+      <c r="BL139" s="16">
+        <v>18093</v>
+      </c>
+      <c r="BM139" s="16">
+        <v>4790</v>
+      </c>
+      <c r="BN139" s="16">
+        <v>137</v>
+      </c>
+      <c r="BO139" s="16">
+        <v>5665</v>
+      </c>
+      <c r="BP139" s="16">
+        <v>125355</v>
+      </c>
+      <c r="BQ139" s="16">
+        <v>119286</v>
+      </c>
+      <c r="BR139" s="16">
+        <v>4142</v>
+      </c>
+      <c r="BS139" s="16">
+        <v>1021</v>
+      </c>
+      <c r="BT139" s="16">
+        <v>905</v>
+      </c>
+      <c r="BU139" s="17">
+        <v>57</v>
+      </c>
+      <c r="BV139" s="17">
+        <v>62.4</v>
+      </c>
+      <c r="BW139" s="17">
+        <v>22.9</v>
+      </c>
+      <c r="BX139" s="17">
+        <v>21.3</v>
+      </c>
+      <c r="BY139" s="17">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B5" location="'Series Definitions'!R2C3"/>
@@ -30605,7 +30818,7 @@
         <v>168</v>
       </c>
       <c r="B4" s="27">
-        <v>46252</v>
+        <v>46281</v>
       </c>
     </row>
     <row r="5"/>

</xml_diff>